<commit_message>
Add chocBandit100 & combined key; update grain key
Add Choco pellet dataset and consolidated key files: added Choco pellet behavior/Bandit_100/chocBandit100L1.zip and Combined key.xlsx. Also updated Grain Pellet Feds/GrainPellets_key.xlsx with revisions to the key mapping.
</commit_message>
<xml_diff>
--- a/Grain Pellet Feds/GrainPellets_key.xlsx
+++ b/Grain Pellet Feds/GrainPellets_key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2024059655943/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gowustl-my.sharepoint.com/personal/murrell_wustl_edu/Documents/Documents/Github/PredictingObesity/Grain Pellet Feds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C444797F-24BC-453A-9580-7CB540FA4B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E39D2C31-DCFE-0845-B4EC-D7B6CBDFAEDE}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{C444797F-24BC-453A-9580-7CB540FA4B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{888128B0-E172-45DA-81C2-CCDA1A96234A}"/>
   <bookViews>
-    <workbookView xWindow="5160" yWindow="1160" windowWidth="23500" windowHeight="13800" xr2:uid="{A5DB2D40-6A15-46FE-A2A3-895C8DE6647A}"/>
+    <workbookView minimized="1" xWindow="-27090" yWindow="1320" windowWidth="23505" windowHeight="14445" xr2:uid="{A5DB2D40-6A15-46FE-A2A3-895C8DE6647A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -533,12 +533,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B26F69E1-CE8C-46D9-A66C-773BA5DB87B8}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
@@ -561,9 +561,9 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
@@ -578,15 +578,15 @@
         <v>3</v>
       </c>
       <c r="F2" s="1">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="G2" s="2">
         <v>45859</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1</v>
@@ -601,15 +601,15 @@
         <v>3</v>
       </c>
       <c r="F3" s="1">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="G3" s="2">
         <v>45859</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>1</v>
@@ -624,15 +624,15 @@
         <v>3</v>
       </c>
       <c r="F4" s="1">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="G4" s="2">
         <v>45859</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>1</v>
@@ -647,15 +647,15 @@
         <v>3</v>
       </c>
       <c r="F5" s="1">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="G5" s="2">
         <v>45859</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>1</v>
@@ -670,15 +670,15 @@
         <v>3</v>
       </c>
       <c r="F6" s="1">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="G6" s="2">
         <v>45859</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>1</v>
@@ -693,13 +693,13 @@
         <v>3</v>
       </c>
       <c r="F7" s="1">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="G7" s="2">
         <v>45859</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -722,306 +722,309 @@
         <v>45859</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="1">
+        <v>333</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" s="1">
+        <v>80</v>
+      </c>
+      <c r="G9" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1">
+        <v>333</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F10" s="1">
+        <v>79</v>
+      </c>
+      <c r="G10" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1">
-        <v>333</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F9" s="1">
+      <c r="B11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1">
+        <v>333</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" s="1">
         <v>66</v>
       </c>
-      <c r="G9" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="G11" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="1">
+        <v>333</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="1">
+        <v>71</v>
+      </c>
+      <c r="G12" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1">
+        <v>333</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F13" s="1">
+        <v>68</v>
+      </c>
+      <c r="G13" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>333</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="1">
+        <v>59</v>
+      </c>
+      <c r="G14" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>333</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" s="1">
+        <v>60</v>
+      </c>
+      <c r="G15" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1">
+        <v>333</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" s="1">
+        <v>40</v>
+      </c>
+      <c r="G16" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="1">
+        <v>333</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F17" s="1">
+        <v>62</v>
+      </c>
+      <c r="G17" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1">
+        <v>333</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F18" s="1">
+        <v>63</v>
+      </c>
+      <c r="G18" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C19" s="1">
+        <v>333</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F19" s="1">
+        <v>61</v>
+      </c>
+      <c r="G19" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1">
+        <v>333</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F20" s="1">
+        <v>69</v>
+      </c>
+      <c r="G20" s="2">
+        <v>45859</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" s="1">
-        <v>333</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F10" s="1">
+      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1">
+        <v>333</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F21" s="1">
         <v>67</v>
       </c>
-      <c r="G10" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="1">
-        <v>333</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F11" s="1">
-        <v>68</v>
-      </c>
-      <c r="G11" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C12" s="1">
-        <v>333</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F12" s="1">
-        <v>69</v>
-      </c>
-      <c r="G12" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="1">
-        <v>333</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F13" s="1">
-        <v>70</v>
-      </c>
-      <c r="G13" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" s="1">
-        <v>333</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" s="1">
-        <v>71</v>
-      </c>
-      <c r="G14" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="1">
-        <v>333</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F15" s="1">
-        <v>72</v>
-      </c>
-      <c r="G15" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1">
-        <v>333</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F16" s="1">
-        <v>74</v>
-      </c>
-      <c r="G16" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1">
-        <v>333</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F17" s="1">
-        <v>75</v>
-      </c>
-      <c r="G17" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" s="1">
-        <v>333</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F18" s="1">
-        <v>76</v>
-      </c>
-      <c r="G18" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C19" s="1">
-        <v>333</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F19" s="1">
-        <v>77</v>
-      </c>
-      <c r="G19" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C20" s="1">
-        <v>333</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F20" s="1">
-        <v>79</v>
-      </c>
-      <c r="G20" s="2">
-        <v>45859</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C21" s="1">
-        <v>333</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F21" s="1">
-        <v>80</v>
-      </c>
       <c r="G21" s="2">
         <v>45859</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G21">
+    <sortCondition ref="A1:A21"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>